<commit_message>
Fixed the bug/caveat about multiple entries in the same cache level being modified in the same access. This is now correctly reflected.
</commit_message>
<xml_diff>
--- a/test/tcs04_LRU_TextProblem_WT/output.xlsx
+++ b/test/tcs04_LRU_TextProblem_WT/output.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.78" customWidth="1" min="1" max="1"/>
@@ -548,369 +548,378 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28.8" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3" ht="28.8" customHeight="1"/>
+    <row r="4" ht="28.8" customHeight="1">
+      <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>20,200
 (V:T, D:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:T, TS:1, LAT:1)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>20,200
 (V:T, D:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:T, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>0,0
 (V:F, D:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>0,0
 (V:F, D:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28.8" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="5" ht="28.8" customHeight="1"/>
+    <row r="6" ht="28.8" customHeight="1">
+      <c r="A6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:T, TS:2, LAT:2)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>20,200
 (V:T, D:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:F, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:T, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>0,0
 (V:F, D:F, MCA:F, TS:0, LAT:0)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="28.8" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="7" ht="28.8" customHeight="1"/>
+    <row r="8" ht="28.8" customHeight="1">
+      <c r="A8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:2, LAT:2)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:T, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>20,200
 (V:T, D:F, MCA:F, TS:1, LAT:1)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:F, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:T, TS:7, LAT:7)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="28.8" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="9" ht="28.8" customHeight="1"/>
+    <row r="10" ht="28.8" customHeight="1">
+      <c r="A10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:T, TS:4, LAT:4)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:T, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>21,300
 (V:T, D:F, MCA:F, TS:3, LAT:3)</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28.8" customHeight="1">
-      <c r="A7" s="2" t="n">
+    <row r="11" ht="28.8" customHeight="1"/>
+    <row r="12" ht="28.8" customHeight="1">
+      <c r="A12" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:4, LAT:4)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:T, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:T, TS:11, LAT:11)</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28.8" customHeight="1">
-      <c r="A8" s="2" t="n">
+    <row r="13" ht="28.8" customHeight="1"/>
+    <row r="14" ht="28.8" customHeight="1">
+      <c r="A14" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:T, TS:6, LAT:6)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:F, TS:5, LAT:5)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:5, LAT:12)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28.8" customHeight="1">
-      <c r="A9" s="2" t="n">
+    <row r="15" ht="28.8" customHeight="1"/>
+    <row r="16" ht="28.8" customHeight="1">
+      <c r="A16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:6, LAT:6)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:T, TS:7, LAT:7)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>22,400
 (V:T, D:F, MCA:F, TS:5, LAT:12)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:13)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28.8" customHeight="1">
-      <c r="A10" s="2" t="n">
+    <row r="17" ht="28.8" customHeight="1"/>
+    <row r="18" ht="28.8" customHeight="1">
+      <c r="A18" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>22,401
 (V:T, D:F, MCA:T, TS:8, LAT:8)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:7)</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>22,401
 (V:T, D:F, MCA:T, TS:14, LAT:14)</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>23,500
 (V:T, D:F, MCA:F, TS:7, LAT:13)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28.8" customHeight="1">
-      <c r="A11" s="2" t="n">
+    <row r="19" ht="28.8" customHeight="1"/>
+    <row r="20" ht="28.8" customHeight="1">
+      <c r="A20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>22,401
 (V:T, D:F, MCA:F, TS:8, LAT:8)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>23,501
 (V:T, D:F, MCA:T, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>20,201
 (V:T, D:F, MCA:F, TS:9, LAT:9)</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>21,301
 (V:T, D:F, MCA:F, TS:11, LAT:11)</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>22,401
 (V:T, D:F, MCA:F, TS:14, LAT:14)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>23,501
 (V:T, D:F, MCA:T, TS:15, LAT:15)</t>

</xml_diff>